<commit_message>
#15 @UroojNav ap continue kr len ye issue or Review b kr len BOM
</commit_message>
<xml_diff>
--- a/Deliverables/Orion_Board/BOM/Orion_Board-Altium Gen.xlsx
+++ b/Deliverables/Orion_Board/BOM/Orion_Board-Altium Gen.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24729"/>
-  <workbookPr defaultThemeVersion="166925"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="7" rupBuild="14420"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark\SH-CircuitCorrections\Deliverables\Orion_Board\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Github\SH-CircuitCorrections\Deliverables\Orion_Board\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{710054E9-3477-4C2D-B93A-FA77B5812564}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1815" yWindow="300" windowWidth="10335" windowHeight="10620" xr2:uid="{9B25667E-9319-4F73-8973-93AE528D3900}"/>
+    <workbookView xWindow="1815" yWindow="300" windowWidth="10335" windowHeight="10620"/>
   </bookViews>
   <sheets>
     <sheet name="Orion_Board-Altium Gen" sheetId="1" r:id="rId1"/>
@@ -388,7 +387,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -398,7 +397,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -408,6 +407,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFD3D3D3"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -439,7 +444,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -449,6 +454,12 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -764,7 +775,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0BEBDDAD-0719-4199-A8F8-641266ACD1E9}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -795,202 +806,202 @@
       </c>
     </row>
     <row r="2" spans="1:6" ht="30" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="F2" s="4">
+      <c r="F2" s="6">
         <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="30" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="D3" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="E3" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="F3" s="4">
+      <c r="F3" s="6">
         <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="30" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="E4" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="F4" s="4">
+      <c r="F4" s="6">
         <v>8</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="30" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D5" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="E5" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="F5" s="4">
+      <c r="F5" s="6">
         <v>2</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="75" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C6" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="D6" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="E6" s="3" t="s">
+      <c r="E6" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="F6" s="4">
+      <c r="F6" s="6">
         <v>2</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="30" x14ac:dyDescent="0.25">
-      <c r="A7" s="3" t="s">
+      <c r="A7" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="C7" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="D7" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="E7" s="3" t="s">
+      <c r="E7" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="F7" s="4">
+      <c r="F7" s="6">
         <v>2</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="30" x14ac:dyDescent="0.25">
-      <c r="A8" s="3" t="s">
+      <c r="A8" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="B8" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="C8" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="D8" s="3" t="s">
+      <c r="D8" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="E8" s="3" t="s">
+      <c r="E8" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="F8" s="4">
+      <c r="F8" s="6">
         <v>2</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="60" x14ac:dyDescent="0.25">
-      <c r="A9" s="3" t="s">
+      <c r="A9" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="B9" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="C9" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="D9" s="3" t="s">
+      <c r="D9" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="E9" s="3" t="s">
+      <c r="E9" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="F9" s="4">
+      <c r="F9" s="6">
         <v>1</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="30" x14ac:dyDescent="0.25">
-      <c r="A10" s="3" t="s">
+      <c r="A10" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="B10" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="C10" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="D10" s="3" t="s">
+      <c r="D10" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="E10" s="3" t="s">
+      <c r="E10" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="F10" s="4">
+      <c r="F10" s="6">
         <v>2</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="30" x14ac:dyDescent="0.25">
-      <c r="A11" s="3" t="s">
+      <c r="A11" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="B11" s="3" t="s">
+      <c r="B11" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="C11" s="3" t="s">
+      <c r="C11" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="D11" s="3" t="s">
+      <c r="D11" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="E11" s="3" t="s">
+      <c r="E11" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="F11" s="4">
+      <c r="F11" s="6">
         <v>1</v>
       </c>
     </row>
@@ -1115,22 +1126,22 @@
       </c>
     </row>
     <row r="18" spans="1:6" ht="30" x14ac:dyDescent="0.25">
-      <c r="A18" s="3" t="s">
+      <c r="A18" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="B18" s="3" t="s">
+      <c r="B18" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="C18" s="3" t="s">
+      <c r="C18" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="D18" s="3" t="s">
+      <c r="D18" s="5" t="s">
         <v>68</v>
       </c>
-      <c r="E18" s="3" t="s">
+      <c r="E18" s="5" t="s">
         <v>68</v>
       </c>
-      <c r="F18" s="4">
+      <c r="F18" s="6">
         <v>2</v>
       </c>
     </row>
@@ -1155,162 +1166,162 @@
       </c>
     </row>
     <row r="20" spans="1:6" ht="30" x14ac:dyDescent="0.25">
-      <c r="A20" s="3" t="s">
+      <c r="A20" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="B20" s="3" t="s">
+      <c r="B20" s="5" t="s">
         <v>73</v>
       </c>
-      <c r="C20" s="3" t="s">
+      <c r="C20" s="5" t="s">
         <v>74</v>
       </c>
-      <c r="D20" s="3" t="s">
+      <c r="D20" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="E20" s="3" t="s">
+      <c r="E20" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="F20" s="4">
+      <c r="F20" s="6">
         <v>4</v>
       </c>
     </row>
     <row r="21" spans="1:6" ht="45" x14ac:dyDescent="0.25">
-      <c r="A21" s="3" t="s">
+      <c r="A21" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="B21" s="3" t="s">
+      <c r="B21" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="C21" s="3" t="s">
+      <c r="C21" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="D21" s="3" t="s">
+      <c r="D21" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="E21" s="3" t="s">
+      <c r="E21" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="F21" s="4">
+      <c r="F21" s="6">
         <v>1</v>
       </c>
     </row>
     <row r="22" spans="1:6" ht="90" x14ac:dyDescent="0.25">
-      <c r="A22" s="3" t="s">
+      <c r="A22" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="B22" s="3" t="s">
+      <c r="B22" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="C22" s="3" t="s">
+      <c r="C22" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="D22" s="3" t="s">
+      <c r="D22" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="E22" s="3" t="s">
+      <c r="E22" s="5" t="s">
         <v>86</v>
       </c>
-      <c r="F22" s="4">
+      <c r="F22" s="6">
         <v>9</v>
       </c>
     </row>
     <row r="23" spans="1:6" ht="30" x14ac:dyDescent="0.25">
-      <c r="A23" s="3" t="s">
+      <c r="A23" s="5" t="s">
         <v>87</v>
       </c>
-      <c r="B23" s="3" t="s">
+      <c r="B23" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="C23" s="3" t="s">
+      <c r="C23" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="D23" s="3" t="s">
+      <c r="D23" s="5" t="s">
         <v>90</v>
       </c>
-      <c r="E23" s="3" t="s">
+      <c r="E23" s="5" t="s">
         <v>91</v>
       </c>
-      <c r="F23" s="4">
+      <c r="F23" s="6">
         <v>2</v>
       </c>
     </row>
     <row r="24" spans="1:6" ht="30" x14ac:dyDescent="0.25">
-      <c r="A24" s="3" t="s">
+      <c r="A24" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="B24" s="3" t="s">
+      <c r="B24" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="C24" s="3" t="s">
+      <c r="C24" s="5" t="s">
         <v>94</v>
       </c>
-      <c r="D24" s="3" t="s">
+      <c r="D24" s="5" t="s">
         <v>90</v>
       </c>
-      <c r="E24" s="3" t="s">
+      <c r="E24" s="5" t="s">
         <v>95</v>
       </c>
-      <c r="F24" s="4">
+      <c r="F24" s="6">
         <v>2</v>
       </c>
     </row>
     <row r="25" spans="1:6" ht="30" x14ac:dyDescent="0.25">
-      <c r="A25" s="3" t="s">
+      <c r="A25" s="5" t="s">
         <v>96</v>
       </c>
-      <c r="B25" s="3" t="s">
+      <c r="B25" s="5" t="s">
         <v>97</v>
       </c>
-      <c r="C25" s="3" t="s">
+      <c r="C25" s="5" t="s">
         <v>98</v>
       </c>
-      <c r="D25" s="3" t="s">
+      <c r="D25" s="5" t="s">
         <v>90</v>
       </c>
-      <c r="E25" s="3" t="s">
+      <c r="E25" s="5" t="s">
         <v>99</v>
       </c>
-      <c r="F25" s="4">
+      <c r="F25" s="6">
         <v>2</v>
       </c>
     </row>
     <row r="26" spans="1:6" ht="60" x14ac:dyDescent="0.25">
-      <c r="A26" s="3" t="s">
+      <c r="A26" s="5" t="s">
         <v>100</v>
       </c>
-      <c r="B26" s="3" t="s">
+      <c r="B26" s="5" t="s">
         <v>101</v>
       </c>
-      <c r="C26" s="3" t="s">
+      <c r="C26" s="5" t="s">
         <v>102</v>
       </c>
-      <c r="D26" s="3" t="s">
+      <c r="D26" s="5" t="s">
         <v>100</v>
       </c>
-      <c r="E26" s="3" t="s">
+      <c r="E26" s="5" t="s">
         <v>100</v>
       </c>
-      <c r="F26" s="4">
+      <c r="F26" s="6">
         <v>5</v>
       </c>
     </row>
     <row r="27" spans="1:6" ht="30" x14ac:dyDescent="0.25">
-      <c r="A27" s="3" t="s">
+      <c r="A27" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="B27" s="3" t="s">
+      <c r="B27" s="5" t="s">
         <v>104</v>
       </c>
-      <c r="C27" s="3" t="s">
+      <c r="C27" s="5" t="s">
         <v>105</v>
       </c>
-      <c r="D27" s="3" t="s">
+      <c r="D27" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="E27" s="3" t="s">
+      <c r="E27" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="F27" s="4">
+      <c r="F27" s="6">
         <v>1</v>
       </c>
     </row>

</xml_diff>